<commit_message>
Update human verification spreadsheets
</commit_message>
<xml_diff>
--- a/human_verification/issue_type_5reviewers_215.xlsx
+++ b/human_verification/issue_type_5reviewers_215.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\15039\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\15039\Desktop\ICSE_27_SWE-design\human_verification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E193D86-339A-4F4F-8666-43A0242A8816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78BBCE7F-2530-472A-B860-8784F07BA66E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="41130" yWindow="2470" windowWidth="16200" windowHeight="9310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3981" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3981" uniqueCount="337">
   <si>
     <t>id</t>
   </si>
@@ -1205,6 +1205,66 @@
   </si>
   <si>
     <t>None: 131; Temporary Solution &amp; Workaround: 21; Contract Violation &amp; Robustness Issues: 13; Inefficient Design &amp; Performance Issues: 10; Logical, Semantic, and Algorithmic Strategy Issues: 9; Coupling, Responsibility and Layering Violation: 6; Incomplete Design: 6; Resource Management Issues: 5; Legacy Compatibility &amp; Migration Issues: 3; Security &amp; Authorization Issues: 3; Build, Environment, and Portability Issues: 2; SSOT &amp; Consistency Issues: 2; Structural Complexity &amp; Readability Issues: 2; Hardcoding &amp; Configurability Issues: 1; Poor Abstraction &amp; Poor Encapsulation: 1</t>
+  </si>
+  <si>
+    <t>Build, Environment, and Portability Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Legacy Compatibility &amp; Migration Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Security &amp; Authorization Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SSOT &amp; Consistency Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Incomplete Design</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Coupling, Responsibility and Layering Violation</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Logical, Semantic, and Algorithmic Strategy Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Inefficient Design &amp; Performance Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Contract Violation &amp; Robustness Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Temporary Solution &amp; Workaround</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Resource Management Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Structural Complexity &amp; Readability Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Poor Abstraction &amp; Poor Encapsulation</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>None</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hardcoding &amp; Configurability Issues</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1758,7 +1818,7 @@
         <v>22</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>24</v>
+        <v>334</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>110</v>
@@ -2106,7 +2166,7 @@
         <v>25</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>19</v>
+        <v>327</v>
       </c>
       <c r="M9" s="2" t="s">
         <v>25</v>
@@ -2147,7 +2207,7 @@
         <v>23</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>18</v>
+        <v>332</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>29</v>
@@ -2159,7 +2219,7 @@
         <v>29</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>19</v>
+        <v>332</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>29</v>
@@ -2265,7 +2325,7 @@
         <v>22</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>19</v>
+        <v>329</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>22</v>
@@ -2401,7 +2461,7 @@
         <v>23</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>19</v>
+        <v>327</v>
       </c>
       <c r="M14" s="2" t="s">
         <v>23</v>
@@ -2442,7 +2502,7 @@
         <v>31</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>19</v>
+        <v>327</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>31</v>
@@ -2584,7 +2644,7 @@
         <v>23</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>31</v>
+        <v>335</v>
       </c>
       <c r="O17" s="2" t="s">
         <v>139</v>
@@ -2678,7 +2738,7 @@
         <v>23</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>29</v>
+        <v>330</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>23</v>
@@ -2808,7 +2868,7 @@
         <v>27</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>41</v>
+        <v>335</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>27</v>
@@ -3038,7 +3098,7 @@
         <v>27</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>27</v>
@@ -3150,7 +3210,7 @@
         <v>44</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>94</v>
@@ -3168,7 +3228,7 @@
         <v>94</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>31</v>
+        <v>331</v>
       </c>
       <c r="M27" s="2" t="s">
         <v>94</v>
@@ -3386,7 +3446,7 @@
         <v>31</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>31</v>
@@ -3463,7 +3523,7 @@
         <v>23</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>19</v>
+        <v>324</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>23</v>
@@ -3622,7 +3682,7 @@
         <v>31</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>22</v>
+        <v>332</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>31</v>
@@ -3699,7 +3759,7 @@
         <v>29</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>23</v>
+        <v>335</v>
       </c>
       <c r="M36" s="2" t="s">
         <v>29</v>
@@ -3740,7 +3800,7 @@
         <v>31</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>19</v>
+        <v>330</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>31</v>
@@ -3758,7 +3818,7 @@
         <v>31</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>22</v>
+        <v>330</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>23</v>
@@ -3817,7 +3877,7 @@
         <v>22</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>31</v>
+        <v>335</v>
       </c>
       <c r="M38" s="2" t="s">
         <v>31</v>
@@ -3917,7 +3977,7 @@
         <v>27</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>22</v>
+        <v>335</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>31</v>
@@ -4000,7 +4060,7 @@
         <v>24</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>36</v>
+        <v>335</v>
       </c>
       <c r="O41" s="2" t="s">
         <v>193</v>
@@ -4041,7 +4101,7 @@
         <v>23</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>27</v>
+        <v>332</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>23</v>
@@ -4053,7 +4113,7 @@
         <v>23</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>19</v>
+        <v>332</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>29</v>
@@ -4153,7 +4213,7 @@
         <v>31</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>23</v>
+        <v>335</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>31</v>
@@ -4342,7 +4402,7 @@
         <v>26</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="K47" s="2" t="s">
         <v>25</v>
@@ -4407,7 +4467,7 @@
         <v>44</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>51</v>
+        <v>335</v>
       </c>
       <c r="M48" s="2" t="s">
         <v>27</v>
@@ -4460,7 +4520,7 @@
         <v>31</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>31</v>
@@ -4549,7 +4609,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="51" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>3850</v>
       </c>
@@ -4584,7 +4644,7 @@
         <v>31</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="M51" s="2" t="s">
         <v>31</v>
@@ -4631,7 +4691,7 @@
         <v>24</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>19</v>
+        <v>328</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>24</v>
@@ -4696,7 +4756,7 @@
         <v>25</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>19</v>
+        <v>326</v>
       </c>
       <c r="K53" s="2" t="s">
         <v>25</v>
@@ -4814,7 +4874,7 @@
         <v>31</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="K55" s="2" t="s">
         <v>31</v>
@@ -5174,7 +5234,7 @@
         <v>24</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>22</v>
+        <v>335</v>
       </c>
       <c r="M61" s="2" t="s">
         <v>24</v>
@@ -5339,7 +5399,7 @@
         <v>31</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>19</v>
+        <v>328</v>
       </c>
       <c r="I64" s="2" t="s">
         <v>31</v>
@@ -5410,7 +5470,7 @@
         <v>23</v>
       </c>
       <c r="L65" s="2" t="s">
-        <v>19</v>
+        <v>329</v>
       </c>
       <c r="M65" s="2" t="s">
         <v>23</v>
@@ -5469,7 +5529,7 @@
         <v>29</v>
       </c>
       <c r="L66" s="2" t="s">
-        <v>19</v>
+        <v>325</v>
       </c>
       <c r="M66" s="2" t="s">
         <v>29</v>
@@ -5764,7 +5824,7 @@
         <v>23</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="M71" s="2" t="s">
         <v>23</v>
@@ -5882,7 +5942,7 @@
         <v>22</v>
       </c>
       <c r="L73" s="2" t="s">
-        <v>24</v>
+        <v>335</v>
       </c>
       <c r="M73" s="2" t="s">
         <v>22</v>
@@ -5965,7 +6025,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="75" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>7752</v>
       </c>
@@ -5988,7 +6048,7 @@
         <v>18</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="I75" s="2" t="s">
         <v>18</v>
@@ -6041,7 +6101,7 @@
         <v>22</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>19</v>
+        <v>329</v>
       </c>
       <c r="G76" s="2" t="s">
         <v>22</v>
@@ -6177,7 +6237,7 @@
         <v>25</v>
       </c>
       <c r="L78" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="M78" s="2" t="s">
         <v>25</v>
@@ -6230,7 +6290,7 @@
         <v>27</v>
       </c>
       <c r="J79" s="2" t="s">
-        <v>22</v>
+        <v>335</v>
       </c>
       <c r="K79" s="2" t="s">
         <v>27</v>
@@ -6336,7 +6396,7 @@
         <v>27</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>41</v>
+        <v>335</v>
       </c>
       <c r="G81" s="2" t="s">
         <v>27</v>
@@ -6413,7 +6473,7 @@
         <v>29</v>
       </c>
       <c r="L82" s="2" t="s">
-        <v>19</v>
+        <v>329</v>
       </c>
       <c r="M82" s="2" t="s">
         <v>29</v>
@@ -6590,7 +6650,7 @@
         <v>29</v>
       </c>
       <c r="L85" s="2" t="s">
-        <v>19</v>
+        <v>330</v>
       </c>
       <c r="M85" s="2" t="s">
         <v>29</v>
@@ -6714,7 +6774,7 @@
         <v>27</v>
       </c>
       <c r="N87" s="2" t="s">
-        <v>31</v>
+        <v>335</v>
       </c>
       <c r="O87" s="2" t="s">
         <v>141</v>
@@ -6773,7 +6833,7 @@
         <v>29</v>
       </c>
       <c r="N88" s="2" t="s">
-        <v>27</v>
+        <v>329</v>
       </c>
       <c r="O88" s="2" t="s">
         <v>171</v>
@@ -6873,7 +6933,7 @@
         <v>23</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>19</v>
+        <v>327</v>
       </c>
       <c r="I90" s="2" t="s">
         <v>23</v>
@@ -7127,7 +7187,7 @@
         <v>31</v>
       </c>
       <c r="N94" s="2" t="s">
-        <v>22</v>
+        <v>335</v>
       </c>
       <c r="O94" s="2" t="s">
         <v>168</v>
@@ -7168,7 +7228,7 @@
         <v>31</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="I95" s="2" t="s">
         <v>31</v>
@@ -7416,7 +7476,7 @@
         <v>27</v>
       </c>
       <c r="L99" s="2" t="s">
-        <v>19</v>
+        <v>326</v>
       </c>
       <c r="M99" s="2" t="s">
         <v>27</v>
@@ -7475,7 +7535,7 @@
         <v>22</v>
       </c>
       <c r="L100" s="2" t="s">
-        <v>19</v>
+        <v>329</v>
       </c>
       <c r="M100" s="2" t="s">
         <v>22</v>
@@ -7499,7 +7559,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="101" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
         <v>2024</v>
       </c>
@@ -7528,7 +7588,7 @@
         <v>31</v>
       </c>
       <c r="J101" s="2" t="s">
-        <v>23</v>
+        <v>335</v>
       </c>
       <c r="K101" s="2" t="s">
         <v>31</v>
@@ -7693,7 +7753,7 @@
         <v>22</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>24</v>
+        <v>335</v>
       </c>
       <c r="G104" s="2" t="s">
         <v>22</v>
@@ -7752,7 +7812,7 @@
         <v>31</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="G105" s="2" t="s">
         <v>31</v>
@@ -8148,7 +8208,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="112" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
         <v>3960</v>
       </c>
@@ -8189,7 +8249,7 @@
         <v>31</v>
       </c>
       <c r="N112" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="O112" s="2" t="s">
         <v>122</v>
@@ -8242,7 +8302,7 @@
         <v>23</v>
       </c>
       <c r="L113" s="2" t="s">
-        <v>29</v>
+        <v>335</v>
       </c>
       <c r="M113" s="2" t="s">
         <v>23</v>
@@ -8301,7 +8361,7 @@
         <v>22</v>
       </c>
       <c r="L114" s="2" t="s">
-        <v>24</v>
+        <v>335</v>
       </c>
       <c r="M114" s="2" t="s">
         <v>22</v>
@@ -8413,7 +8473,7 @@
         <v>27</v>
       </c>
       <c r="J116" s="2" t="s">
-        <v>23</v>
+        <v>335</v>
       </c>
       <c r="K116" s="2" t="s">
         <v>31</v>
@@ -8543,7 +8603,7 @@
         <v>29</v>
       </c>
       <c r="N118" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="O118" s="2" t="s">
         <v>252</v>
@@ -8655,7 +8715,7 @@
         <v>22</v>
       </c>
       <c r="L120" s="2" t="s">
-        <v>27</v>
+        <v>326</v>
       </c>
       <c r="M120" s="2" t="s">
         <v>22</v>
@@ -8702,7 +8762,7 @@
         <v>23</v>
       </c>
       <c r="H121" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="I121" s="2" t="s">
         <v>31</v>
@@ -8838,7 +8898,7 @@
         <v>44</v>
       </c>
       <c r="N123" s="2" t="s">
-        <v>51</v>
+        <v>335</v>
       </c>
       <c r="O123" s="2" t="s">
         <v>165</v>
@@ -8891,7 +8951,7 @@
         <v>31</v>
       </c>
       <c r="L124" s="2" t="s">
-        <v>22</v>
+        <v>335</v>
       </c>
       <c r="M124" s="2" t="s">
         <v>27</v>
@@ -8950,7 +9010,7 @@
         <v>31</v>
       </c>
       <c r="L125" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="M125" s="2" t="s">
         <v>31</v>
@@ -9068,7 +9128,7 @@
         <v>44</v>
       </c>
       <c r="L127" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="M127" s="2" t="s">
         <v>44</v>
@@ -9151,7 +9211,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="129" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A129" s="2">
         <v>5185</v>
       </c>
@@ -9180,7 +9240,7 @@
         <v>18</v>
       </c>
       <c r="J129" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="K129" s="2" t="s">
         <v>18</v>
@@ -9210,7 +9270,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="130" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A130" s="2">
         <v>5257</v>
       </c>
@@ -9251,7 +9311,7 @@
         <v>31</v>
       </c>
       <c r="N130" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="O130" s="2" t="s">
         <v>122</v>
@@ -9505,7 +9565,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="135" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A135" s="2">
         <v>1089</v>
       </c>
@@ -9522,7 +9582,7 @@
         <v>31</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>23</v>
+        <v>335</v>
       </c>
       <c r="G135" s="2" t="s">
         <v>31</v>
@@ -9646,7 +9706,7 @@
         <v>25</v>
       </c>
       <c r="H137" s="2" t="s">
-        <v>51</v>
+        <v>335</v>
       </c>
       <c r="I137" s="2" t="s">
         <v>25</v>
@@ -10065,7 +10125,7 @@
         <v>100</v>
       </c>
       <c r="J144" s="2" t="s">
-        <v>24</v>
+        <v>333</v>
       </c>
       <c r="K144" s="2" t="s">
         <v>100</v>
@@ -10242,7 +10302,7 @@
         <v>44</v>
       </c>
       <c r="J147" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="K147" s="2" t="s">
         <v>44</v>
@@ -10272,7 +10332,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="148" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A148" s="2">
         <v>3931</v>
       </c>
@@ -10289,7 +10349,7 @@
         <v>31</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="G148" s="2" t="s">
         <v>31</v>
@@ -10348,7 +10408,7 @@
         <v>31</v>
       </c>
       <c r="F149" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="G149" s="2" t="s">
         <v>23</v>
@@ -10508,7 +10568,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="152" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A152" s="2">
         <v>4668</v>
       </c>
@@ -10537,7 +10597,7 @@
         <v>31</v>
       </c>
       <c r="J152" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="K152" s="2" t="s">
         <v>31</v>
@@ -10608,7 +10668,7 @@
         <v>31</v>
       </c>
       <c r="N153" s="2" t="s">
-        <v>22</v>
+        <v>335</v>
       </c>
       <c r="O153" s="2" t="s">
         <v>200</v>
@@ -10649,7 +10709,7 @@
         <v>27</v>
       </c>
       <c r="H154" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="I154" s="2" t="s">
         <v>27</v>
@@ -10779,7 +10839,7 @@
         <v>31</v>
       </c>
       <c r="L156" s="2" t="s">
-        <v>19</v>
+        <v>330</v>
       </c>
       <c r="M156" s="2" t="s">
         <v>31</v>
@@ -10826,7 +10886,7 @@
         <v>27</v>
       </c>
       <c r="H157" s="2" t="s">
-        <v>19</v>
+        <v>328</v>
       </c>
       <c r="I157" s="2" t="s">
         <v>27</v>
@@ -10938,7 +10998,7 @@
         <v>44</v>
       </c>
       <c r="F159" s="2" t="s">
-        <v>27</v>
+        <v>331</v>
       </c>
       <c r="G159" s="2" t="s">
         <v>44</v>
@@ -11133,7 +11193,7 @@
         <v>31</v>
       </c>
       <c r="L162" s="2" t="s">
-        <v>22</v>
+        <v>335</v>
       </c>
       <c r="M162" s="2" t="s">
         <v>31</v>
@@ -11310,7 +11370,7 @@
         <v>51</v>
       </c>
       <c r="L165" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="M165" s="2" t="s">
         <v>25</v>
@@ -11363,7 +11423,7 @@
         <v>25</v>
       </c>
       <c r="J166" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="K166" s="2" t="s">
         <v>25</v>
@@ -11410,7 +11470,7 @@
         <v>25</v>
       </c>
       <c r="F167" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="G167" s="2" t="s">
         <v>25</v>
@@ -11540,7 +11600,7 @@
         <v>23</v>
       </c>
       <c r="J169" s="2" t="s">
-        <v>29</v>
+        <v>335</v>
       </c>
       <c r="K169" s="2" t="s">
         <v>23</v>
@@ -11587,7 +11647,7 @@
         <v>31</v>
       </c>
       <c r="F170" s="2" t="s">
-        <v>19</v>
+        <v>323</v>
       </c>
       <c r="G170" s="2" t="s">
         <v>31</v>
@@ -11629,7 +11689,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="171" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A171" s="2">
         <v>4566</v>
       </c>
@@ -11652,7 +11712,7 @@
         <v>31</v>
       </c>
       <c r="H171" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="I171" s="2" t="s">
         <v>31</v>
@@ -11770,7 +11830,7 @@
         <v>44</v>
       </c>
       <c r="H173" s="2" t="s">
-        <v>19</v>
+        <v>331</v>
       </c>
       <c r="I173" s="2" t="s">
         <v>44</v>
@@ -11882,7 +11942,7 @@
         <v>25</v>
       </c>
       <c r="F175" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="G175" s="2" t="s">
         <v>25</v>
@@ -12071,7 +12131,7 @@
         <v>27</v>
       </c>
       <c r="J178" s="2" t="s">
-        <v>22</v>
+        <v>335</v>
       </c>
       <c r="K178" s="2" t="s">
         <v>27</v>
@@ -12177,7 +12237,7 @@
         <v>104</v>
       </c>
       <c r="F180" s="2" t="s">
-        <v>27</v>
+        <v>324</v>
       </c>
       <c r="G180" s="2" t="s">
         <v>104</v>
@@ -12254,7 +12314,7 @@
         <v>27</v>
       </c>
       <c r="L181" s="2" t="s">
-        <v>41</v>
+        <v>335</v>
       </c>
       <c r="M181" s="2" t="s">
         <v>27</v>
@@ -12295,7 +12355,7 @@
         <v>18</v>
       </c>
       <c r="F182" s="2" t="s">
-        <v>29</v>
+        <v>335</v>
       </c>
       <c r="G182" s="2" t="s">
         <v>18</v>
@@ -12378,7 +12438,7 @@
         <v>27</v>
       </c>
       <c r="N183" s="2" t="s">
-        <v>19</v>
+        <v>325</v>
       </c>
       <c r="O183" s="2" t="s">
         <v>141</v>
@@ -12608,7 +12668,7 @@
         <v>18</v>
       </c>
       <c r="L187" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="M187" s="2" t="s">
         <v>18</v>
@@ -12667,7 +12727,7 @@
         <v>23</v>
       </c>
       <c r="L188" s="2" t="s">
-        <v>29</v>
+        <v>335</v>
       </c>
       <c r="M188" s="2" t="s">
         <v>23</v>
@@ -12708,7 +12768,7 @@
         <v>23</v>
       </c>
       <c r="F189" s="2" t="s">
-        <v>19</v>
+        <v>322</v>
       </c>
       <c r="G189" s="2" t="s">
         <v>23</v>
@@ -12785,7 +12845,7 @@
         <v>23</v>
       </c>
       <c r="L190" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="M190" s="2" t="s">
         <v>27</v>
@@ -12891,7 +12951,7 @@
         <v>23</v>
       </c>
       <c r="H192" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="I192" s="2" t="s">
         <v>23</v>
@@ -13068,7 +13128,7 @@
         <v>23</v>
       </c>
       <c r="H195" s="2" t="s">
-        <v>31</v>
+        <v>325</v>
       </c>
       <c r="I195" s="2" t="s">
         <v>27</v>
@@ -13080,7 +13140,7 @@
         <v>31</v>
       </c>
       <c r="L195" s="2" t="s">
-        <v>19</v>
+        <v>325</v>
       </c>
       <c r="M195" s="2" t="s">
         <v>23</v>
@@ -13198,7 +13258,7 @@
         <v>27</v>
       </c>
       <c r="L197" s="2" t="s">
-        <v>41</v>
+        <v>335</v>
       </c>
       <c r="M197" s="2" t="s">
         <v>27</v>
@@ -13363,7 +13423,7 @@
         <v>23</v>
       </c>
       <c r="H200" s="2" t="s">
-        <v>19</v>
+        <v>323</v>
       </c>
       <c r="I200" s="2" t="s">
         <v>23</v>
@@ -13440,7 +13500,7 @@
         <v>23</v>
       </c>
       <c r="N201" s="2" t="s">
-        <v>29</v>
+        <v>335</v>
       </c>
       <c r="O201" s="2" t="s">
         <v>139</v>
@@ -13481,7 +13541,7 @@
         <v>23</v>
       </c>
       <c r="H202" s="2" t="s">
-        <v>27</v>
+        <v>335</v>
       </c>
       <c r="I202" s="2" t="s">
         <v>23</v>
@@ -13540,7 +13600,7 @@
         <v>23</v>
       </c>
       <c r="H203" s="2" t="s">
-        <v>19</v>
+        <v>336</v>
       </c>
       <c r="I203" s="2" t="s">
         <v>23</v>
@@ -13652,7 +13712,7 @@
         <v>31</v>
       </c>
       <c r="F205" s="2" t="s">
-        <v>23</v>
+        <v>335</v>
       </c>
       <c r="G205" s="2" t="s">
         <v>31</v>
@@ -13871,7 +13931,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="209" spans="1:19" ht="27" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A209" s="2">
         <v>8687</v>
       </c>
@@ -13894,7 +13954,7 @@
         <v>31</v>
       </c>
       <c r="H209" s="2" t="s">
-        <v>23</v>
+        <v>335</v>
       </c>
       <c r="I209" s="2" t="s">
         <v>31</v>
@@ -14012,7 +14072,7 @@
         <v>31</v>
       </c>
       <c r="H211" s="2" t="s">
-        <v>24</v>
+        <v>335</v>
       </c>
       <c r="I211" s="2" t="s">
         <v>22</v>
@@ -14142,7 +14202,7 @@
         <v>18</v>
       </c>
       <c r="L213" s="2" t="s">
-        <v>22</v>
+        <v>335</v>
       </c>
       <c r="M213" s="2" t="s">
         <v>18</v>
@@ -14260,7 +14320,7 @@
         <v>18</v>
       </c>
       <c r="L215" s="2" t="s">
-        <v>29</v>
+        <v>335</v>
       </c>
       <c r="M215" s="2" t="s">
         <v>29</v>

</xml_diff>